<commit_message>
feat: update aux crawl 12/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -933,7 +933,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1225,7 +1225,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -9961,7 +9961,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -10657,7 +10657,7 @@
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="C14" s="59" t="inlineStr">
@@ -10666,21 +10666,39 @@
         </is>
       </c>
       <c r="D14" s="168" t="n">
-        <v>46277.02385240931</v>
-      </c>
-      <c r="E14" s="168" t="n"/>
+        <v>46277.02385240741</v>
+      </c>
+      <c r="E14" s="168" t="n">
+        <v>46277.83505616898</v>
+      </c>
       <c r="F14" s="169">
         <f>IF(AND(D14&lt;&gt;"",E14&lt;&gt;""),(E14-D14)*24,"")</f>
         <v/>
       </c>
-      <c r="G14" s="170" t="n"/>
-      <c r="H14" s="170" t="n"/>
-      <c r="I14" s="170" t="n"/>
-      <c r="J14" s="170" t="n"/>
-      <c r="K14" s="170" t="n"/>
-      <c r="L14" s="170" t="n"/>
-      <c r="M14" s="170" t="n"/>
-      <c r="N14" s="170" t="n"/>
+      <c r="G14" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H14" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I14" s="170" t="n">
+        <v>3175</v>
+      </c>
+      <c r="J14" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="170" t="n">
+        <v>315</v>
+      </c>
+      <c r="L14" s="170" t="n">
+        <v>30</v>
+      </c>
+      <c r="M14" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N14" s="170" t="n">
+        <v>29730</v>
+      </c>
       <c r="O14" s="170" t="n">
         <v>10</v>
       </c>
@@ -10691,7 +10709,7 @@
       </c>
       <c r="Q14" s="59" t="inlineStr">
         <is>
-          <t>Scheduled durable run; save_artifacts=false</t>
+          <t>Scheduled run 11 terminal</t>
         </is>
       </c>
     </row>
@@ -10701,11 +10719,17 @@
       </c>
       <c r="B15" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C15" s="59" t="n"/>
-      <c r="D15" s="168" t="n"/>
+          <t>Đang chạy</t>
+        </is>
+      </c>
+      <c r="C15" s="59" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D15" s="168" t="n">
+        <v>46277.73217592593</v>
+      </c>
       <c r="E15" s="168" t="n"/>
       <c r="F15" s="169">
         <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),(E15-D15)*24,"")</f>
@@ -10727,7 +10751,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q15" s="59" t="n"/>
+      <c r="Q15" s="59" t="inlineStr">
+        <is>
+          <t>Recovered monitor cho scheduled run 12; không tạo run thay thế</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="167" t="n">
@@ -13406,7 +13434,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -18578,7 +18606,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -21818,7 +21846,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -22530,7 +22558,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -23020,7 +23048,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat: updare aux crawl 13/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -933,7 +933,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1225,7 +1225,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -9961,7 +9961,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -10719,7 +10719,7 @@
       </c>
       <c r="B15" s="59" t="inlineStr">
         <is>
-          <t>Đang chạy</t>
+          <t>Hoàn thành có lỗi</t>
         </is>
       </c>
       <c r="C15" s="59" t="inlineStr">
@@ -10730,19 +10730,37 @@
       <c r="D15" s="168" t="n">
         <v>46277.73217592593</v>
       </c>
-      <c r="E15" s="168" t="n"/>
+      <c r="E15" s="168" t="n">
+        <v>46278.79689062534</v>
+      </c>
       <c r="F15" s="169">
         <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),(E15-D15)*24,"")</f>
         <v/>
       </c>
-      <c r="G15" s="170" t="n"/>
-      <c r="H15" s="170" t="n"/>
-      <c r="I15" s="170" t="n"/>
-      <c r="J15" s="170" t="n"/>
-      <c r="K15" s="170" t="n"/>
-      <c r="L15" s="170" t="n"/>
-      <c r="M15" s="170" t="n"/>
-      <c r="N15" s="170" t="n"/>
+      <c r="G15" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H15" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I15" s="170" t="n">
+        <v>3175</v>
+      </c>
+      <c r="J15" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="170" t="n">
+        <v>315</v>
+      </c>
+      <c r="L15" s="170" t="n">
+        <v>30</v>
+      </c>
+      <c r="M15" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N15" s="170" t="n">
+        <v>29379</v>
+      </c>
       <c r="O15" s="170" t="n">
         <v>10</v>
       </c>
@@ -10753,7 +10771,7 @@
       </c>
       <c r="Q15" s="59" t="inlineStr">
         <is>
-          <t>Recovered monitor cho scheduled run 12; không tạo run thay thế</t>
+          <t>Scheduled run 12 terminal</t>
         </is>
       </c>
     </row>
@@ -13434,7 +13452,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -18606,7 +18624,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I93"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -21846,7 +21864,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -22558,7 +22576,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -23048,7 +23066,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat: update aux crawl 19/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -10731,7 +10731,7 @@
         <v>46277.73217592593</v>
       </c>
       <c r="E15" s="168" t="n">
-        <v>46278.79689062534</v>
+        <v>46278.796890625</v>
       </c>
       <c r="F15" s="169">
         <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),(E15-D15)*24,"")</f>
@@ -10781,19 +10781,33 @@
       </c>
       <c r="B16" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C16" s="59" t="n"/>
-      <c r="D16" s="168" t="n"/>
-      <c r="E16" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D16" s="168" t="n">
+        <v>46278.72856481482</v>
+      </c>
+      <c r="E16" s="168" t="n">
+        <v>46279.90620111111</v>
+      </c>
       <c r="F16" s="169">
         <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),(E16-D16)*24,"")</f>
         <v/>
       </c>
-      <c r="G16" s="170" t="n"/>
-      <c r="H16" s="170" t="n"/>
-      <c r="I16" s="170" t="n"/>
+      <c r="G16" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H16" s="170" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="170" t="n">
+        <v>2</v>
+      </c>
       <c r="J16" s="170" t="n"/>
       <c r="K16" s="170" t="n"/>
       <c r="L16" s="170" t="n"/>
@@ -10807,7 +10821,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q16" s="59" t="n"/>
+      <c r="Q16" s="59" t="inlineStr">
+        <is>
+          <t>Bỏ qua theo yêu cầu người dùng; dừng run 13 sau 2/3540 item. Ngày kế tiếp chạy độc lập.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="167" t="n">
@@ -10815,24 +10833,48 @@
       </c>
       <c r="B17" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C17" s="59" t="n"/>
-      <c r="D17" s="168" t="n"/>
-      <c r="E17" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C17" s="59" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D17" s="168" t="n">
+        <v>46279.73701388889</v>
+      </c>
+      <c r="E17" s="168" t="n">
+        <v>46280.81530137731</v>
+      </c>
       <c r="F17" s="169">
         <f>IF(AND(D17&lt;&gt;"",E17&lt;&gt;""),(E17-D17)*24,"")</f>
         <v/>
       </c>
-      <c r="G17" s="170" t="n"/>
-      <c r="H17" s="170" t="n"/>
-      <c r="I17" s="170" t="n"/>
-      <c r="J17" s="170" t="n"/>
-      <c r="K17" s="170" t="n"/>
-      <c r="L17" s="170" t="n"/>
-      <c r="M17" s="170" t="n"/>
-      <c r="N17" s="170" t="n"/>
+      <c r="G17" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H17" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I17" s="170" t="n">
+        <v>3152</v>
+      </c>
+      <c r="J17" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="170" t="n">
+        <v>328</v>
+      </c>
+      <c r="L17" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M17" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N17" s="170" t="n">
+        <v>28862</v>
+      </c>
       <c r="O17" s="170" t="n">
         <v>10</v>
       </c>
@@ -10841,7 +10883,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q17" s="59" t="n"/>
+      <c r="Q17" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 14 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="167" t="n">
@@ -10849,24 +10895,48 @@
       </c>
       <c r="B18" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C18" s="59" t="n"/>
-      <c r="D18" s="168" t="n"/>
-      <c r="E18" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C18" s="59" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D18" s="168" t="n">
+        <v>46281.02672401621</v>
+      </c>
+      <c r="E18" s="168" t="n">
+        <v>46281.81371444444</v>
+      </c>
       <c r="F18" s="169">
         <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),(E18-D18)*24,"")</f>
         <v/>
       </c>
-      <c r="G18" s="170" t="n"/>
-      <c r="H18" s="170" t="n"/>
-      <c r="I18" s="170" t="n"/>
-      <c r="J18" s="170" t="n"/>
-      <c r="K18" s="170" t="n"/>
-      <c r="L18" s="170" t="n"/>
-      <c r="M18" s="170" t="n"/>
-      <c r="N18" s="170" t="n"/>
+      <c r="G18" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H18" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I18" s="170" t="n">
+        <v>3170</v>
+      </c>
+      <c r="J18" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="170" t="n">
+        <v>310</v>
+      </c>
+      <c r="L18" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M18" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N18" s="170" t="n">
+        <v>29084</v>
+      </c>
       <c r="O18" s="170" t="n">
         <v>10</v>
       </c>
@@ -10875,7 +10945,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q18" s="59" t="n"/>
+      <c r="Q18" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 15 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="167" t="n">
@@ -10883,24 +10957,48 @@
       </c>
       <c r="B19" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C19" s="59" t="n"/>
-      <c r="D19" s="168" t="n"/>
-      <c r="E19" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D19" s="168" t="n">
+        <v>46282.02266850694</v>
+      </c>
+      <c r="E19" s="168" t="n">
+        <v>46282.78398810185</v>
+      </c>
       <c r="F19" s="169">
         <f>IF(AND(D19&lt;&gt;"",E19&lt;&gt;""),(E19-D19)*24,"")</f>
         <v/>
       </c>
-      <c r="G19" s="170" t="n"/>
-      <c r="H19" s="170" t="n"/>
-      <c r="I19" s="170" t="n"/>
-      <c r="J19" s="170" t="n"/>
-      <c r="K19" s="170" t="n"/>
-      <c r="L19" s="170" t="n"/>
-      <c r="M19" s="170" t="n"/>
-      <c r="N19" s="170" t="n"/>
+      <c r="G19" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H19" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I19" s="170" t="n">
+        <v>3121</v>
+      </c>
+      <c r="J19" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="170" t="n">
+        <v>309</v>
+      </c>
+      <c r="L19" s="170" t="n">
+        <v>90</v>
+      </c>
+      <c r="M19" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N19" s="170" t="n">
+        <v>28229</v>
+      </c>
       <c r="O19" s="170" t="n">
         <v>10</v>
       </c>
@@ -10909,7 +11007,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q19" s="59" t="n"/>
+      <c r="Q19" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 16 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="167" t="n">
@@ -10917,24 +11019,48 @@
       </c>
       <c r="B20" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C20" s="59" t="n"/>
-      <c r="D20" s="168" t="n"/>
-      <c r="E20" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D20" s="168" t="n">
+        <v>46283.02424359954</v>
+      </c>
+      <c r="E20" s="168" t="n">
+        <v>46283.78622950232</v>
+      </c>
       <c r="F20" s="169">
         <f>IF(AND(D20&lt;&gt;"",E20&lt;&gt;""),(E20-D20)*24,"")</f>
         <v/>
       </c>
-      <c r="G20" s="170" t="n"/>
-      <c r="H20" s="170" t="n"/>
-      <c r="I20" s="170" t="n"/>
-      <c r="J20" s="170" t="n"/>
-      <c r="K20" s="170" t="n"/>
-      <c r="L20" s="170" t="n"/>
-      <c r="M20" s="170" t="n"/>
-      <c r="N20" s="170" t="n"/>
+      <c r="G20" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H20" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I20" s="170" t="n">
+        <v>3133</v>
+      </c>
+      <c r="J20" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="170" t="n">
+        <v>307</v>
+      </c>
+      <c r="L20" s="170" t="n">
+        <v>80</v>
+      </c>
+      <c r="M20" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N20" s="170" t="n">
+        <v>28008</v>
+      </c>
       <c r="O20" s="170" t="n">
         <v>10</v>
       </c>
@@ -10943,7 +11069,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q20" s="59" t="n"/>
+      <c r="Q20" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 17 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="167" t="n">
@@ -10951,24 +11081,48 @@
       </c>
       <c r="B21" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C21" s="59" t="n"/>
-      <c r="D21" s="168" t="n"/>
-      <c r="E21" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D21" s="168" t="n">
+        <v>46284.02293990741</v>
+      </c>
+      <c r="E21" s="168" t="n">
+        <v>46284.78843566354</v>
+      </c>
       <c r="F21" s="169">
         <f>IF(AND(D21&lt;&gt;"",E21&lt;&gt;""),(E21-D21)*24,"")</f>
         <v/>
       </c>
-      <c r="G21" s="170" t="n"/>
-      <c r="H21" s="170" t="n"/>
-      <c r="I21" s="170" t="n"/>
-      <c r="J21" s="170" t="n"/>
-      <c r="K21" s="170" t="n"/>
-      <c r="L21" s="170" t="n"/>
-      <c r="M21" s="170" t="n"/>
-      <c r="N21" s="170" t="n"/>
+      <c r="G21" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H21" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I21" s="170" t="n">
+        <v>3156</v>
+      </c>
+      <c r="J21" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="170" t="n">
+        <v>314</v>
+      </c>
+      <c r="L21" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="M21" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N21" s="170" t="n">
+        <v>28398</v>
+      </c>
       <c r="O21" s="170" t="n">
         <v>10</v>
       </c>
@@ -10977,7 +11131,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q21" s="59" t="n"/>
+      <c r="Q21" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 18 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 21/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -11093,7 +11093,7 @@
         <v>46284.02293990741</v>
       </c>
       <c r="E21" s="168" t="n">
-        <v>46284.78843566354</v>
+        <v>46284.78843565972</v>
       </c>
       <c r="F21" s="169">
         <f>IF(AND(D21&lt;&gt;"",E21&lt;&gt;""),(E21-D21)*24,"")</f>
@@ -11143,24 +11143,48 @@
       </c>
       <c r="B22" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C22" s="59" t="n"/>
-      <c r="D22" s="168" t="n"/>
-      <c r="E22" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D22" s="168" t="n">
+        <v>46285.09364074074</v>
+      </c>
+      <c r="E22" s="168" t="n">
+        <v>46285.87094282408</v>
+      </c>
       <c r="F22" s="169">
         <f>IF(AND(D22&lt;&gt;"",E22&lt;&gt;""),(E22-D22)*24,"")</f>
         <v/>
       </c>
-      <c r="G22" s="170" t="n"/>
-      <c r="H22" s="170" t="n"/>
-      <c r="I22" s="170" t="n"/>
-      <c r="J22" s="170" t="n"/>
-      <c r="K22" s="170" t="n"/>
-      <c r="L22" s="170" t="n"/>
-      <c r="M22" s="170" t="n"/>
-      <c r="N22" s="170" t="n"/>
+      <c r="G22" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H22" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I22" s="170" t="n">
+        <v>3140</v>
+      </c>
+      <c r="J22" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="170" t="n">
+        <v>340</v>
+      </c>
+      <c r="L22" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M22" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N22" s="170" t="n">
+        <v>28144</v>
+      </c>
       <c r="O22" s="170" t="n">
         <v>10</v>
       </c>
@@ -11169,7 +11193,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q22" s="59" t="n"/>
+      <c r="Q22" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 19 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="167" t="n">
@@ -11177,24 +11205,48 @@
       </c>
       <c r="B23" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C23" s="59" t="n"/>
-      <c r="D23" s="168" t="n"/>
-      <c r="E23" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D23" s="168" t="n">
+        <v>46286.03120365741</v>
+      </c>
+      <c r="E23" s="168" t="n">
+        <v>46286.80991675532</v>
+      </c>
       <c r="F23" s="169">
         <f>IF(AND(D23&lt;&gt;"",E23&lt;&gt;""),(E23-D23)*24,"")</f>
         <v/>
       </c>
-      <c r="G23" s="170" t="n"/>
-      <c r="H23" s="170" t="n"/>
-      <c r="I23" s="170" t="n"/>
-      <c r="J23" s="170" t="n"/>
-      <c r="K23" s="170" t="n"/>
-      <c r="L23" s="170" t="n"/>
-      <c r="M23" s="170" t="n"/>
-      <c r="N23" s="170" t="n"/>
+      <c r="G23" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H23" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I23" s="170" t="n">
+        <v>3141</v>
+      </c>
+      <c r="J23" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="170" t="n">
+        <v>329</v>
+      </c>
+      <c r="L23" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="M23" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N23" s="170" t="n">
+        <v>27670</v>
+      </c>
       <c r="O23" s="170" t="n">
         <v>10</v>
       </c>
@@ -11203,7 +11255,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q23" s="59" t="n"/>
+      <c r="Q23" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 20 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="167" t="n">

</xml_diff>

<commit_message>
feat: update crawl aux 28/9
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -11341,7 +11341,7 @@
         <v>46288.02336306713</v>
       </c>
       <c r="E25" s="168" t="n">
-        <v>46288.80762244927</v>
+        <v>46288.80762245371</v>
       </c>
       <c r="F25" s="169">
         <f>IF(AND(D25&lt;&gt;"",E25&lt;&gt;""),(E25-D25)*24,"")</f>
@@ -11391,24 +11391,48 @@
       </c>
       <c r="B26" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C26" s="59" t="n"/>
-      <c r="D26" s="168" t="n"/>
-      <c r="E26" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C26" s="59" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D26" s="168" t="n">
+        <v>46289.02872111111</v>
+      </c>
+      <c r="E26" s="168" t="n">
+        <v>46289.82281957176</v>
+      </c>
       <c r="F26" s="169">
         <f>IF(AND(D26&lt;&gt;"",E26&lt;&gt;""),(E26-D26)*24,"")</f>
         <v/>
       </c>
-      <c r="G26" s="170" t="n"/>
-      <c r="H26" s="170" t="n"/>
-      <c r="I26" s="170" t="n"/>
-      <c r="J26" s="170" t="n"/>
-      <c r="K26" s="170" t="n"/>
-      <c r="L26" s="170" t="n"/>
-      <c r="M26" s="170" t="n"/>
-      <c r="N26" s="170" t="n"/>
+      <c r="G26" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H26" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I26" s="170" t="n">
+        <v>3093</v>
+      </c>
+      <c r="J26" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="170" t="n">
+        <v>387</v>
+      </c>
+      <c r="L26" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M26" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N26" s="170" t="n">
+        <v>28165</v>
+      </c>
       <c r="O26" s="170" t="n">
         <v>10</v>
       </c>
@@ -11417,7 +11441,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q26" s="59" t="n"/>
+      <c r="Q26" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 23 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="167" t="n">
@@ -11425,24 +11453,48 @@
       </c>
       <c r="B27" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C27" s="59" t="n"/>
-      <c r="D27" s="168" t="n"/>
-      <c r="E27" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C27" s="59" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D27" s="168" t="n">
+        <v>46290.02340449074</v>
+      </c>
+      <c r="E27" s="168" t="n">
+        <v>46290.91681376157</v>
+      </c>
       <c r="F27" s="169">
         <f>IF(AND(D27&lt;&gt;"",E27&lt;&gt;""),(E27-D27)*24,"")</f>
         <v/>
       </c>
-      <c r="G27" s="170" t="n"/>
-      <c r="H27" s="170" t="n"/>
-      <c r="I27" s="170" t="n"/>
-      <c r="J27" s="170" t="n"/>
-      <c r="K27" s="170" t="n"/>
-      <c r="L27" s="170" t="n"/>
-      <c r="M27" s="170" t="n"/>
-      <c r="N27" s="170" t="n"/>
+      <c r="G27" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H27" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I27" s="170" t="n">
+        <v>3070</v>
+      </c>
+      <c r="J27" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="170" t="n">
+        <v>410</v>
+      </c>
+      <c r="L27" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="M27" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N27" s="170" t="n">
+        <v>27956</v>
+      </c>
       <c r="O27" s="170" t="n">
         <v>10</v>
       </c>
@@ -11451,7 +11503,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q27" s="59" t="n"/>
+      <c r="Q27" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 24 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="167" t="n">
@@ -11459,24 +11515,48 @@
       </c>
       <c r="B28" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C28" s="59" t="n"/>
-      <c r="D28" s="168" t="n"/>
-      <c r="E28" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C28" s="59" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D28" s="168" t="n">
+        <v>46291.0291418287</v>
+      </c>
+      <c r="E28" s="168" t="n">
+        <v>46292.03074357639</v>
+      </c>
       <c r="F28" s="169">
         <f>IF(AND(D28&lt;&gt;"",E28&lt;&gt;""),(E28-D28)*24,"")</f>
         <v/>
       </c>
-      <c r="G28" s="170" t="n"/>
-      <c r="H28" s="170" t="n"/>
-      <c r="I28" s="170" t="n"/>
-      <c r="J28" s="170" t="n"/>
-      <c r="K28" s="170" t="n"/>
-      <c r="L28" s="170" t="n"/>
-      <c r="M28" s="170" t="n"/>
-      <c r="N28" s="170" t="n"/>
+      <c r="G28" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H28" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I28" s="170" t="n">
+        <v>3091</v>
+      </c>
+      <c r="J28" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="170" t="n">
+        <v>339</v>
+      </c>
+      <c r="L28" s="170" t="n">
+        <v>90</v>
+      </c>
+      <c r="M28" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N28" s="170" t="n">
+        <v>29386</v>
+      </c>
       <c r="O28" s="170" t="n">
         <v>10</v>
       </c>
@@ -11485,7 +11565,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q28" s="59" t="n"/>
+      <c r="Q28" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 25 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="167" t="n">
@@ -11493,24 +11577,48 @@
       </c>
       <c r="B29" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C29" s="59" t="n"/>
-      <c r="D29" s="168" t="n"/>
-      <c r="E29" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C29" s="59" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D29" s="168" t="n">
+        <v>46292.01198827547</v>
+      </c>
+      <c r="E29" s="168" t="n">
+        <v>46293.2012952662</v>
+      </c>
       <c r="F29" s="169">
         <f>IF(AND(D29&lt;&gt;"",E29&lt;&gt;""),(E29-D29)*24,"")</f>
         <v/>
       </c>
-      <c r="G29" s="170" t="n"/>
-      <c r="H29" s="170" t="n"/>
-      <c r="I29" s="170" t="n"/>
-      <c r="J29" s="170" t="n"/>
-      <c r="K29" s="170" t="n"/>
-      <c r="L29" s="170" t="n"/>
-      <c r="M29" s="170" t="n"/>
-      <c r="N29" s="170" t="n"/>
+      <c r="G29" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H29" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I29" s="170" t="n">
+        <v>3097</v>
+      </c>
+      <c r="J29" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="170" t="n">
+        <v>323</v>
+      </c>
+      <c r="L29" s="170" t="n">
+        <v>100</v>
+      </c>
+      <c r="M29" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N29" s="170" t="n">
+        <v>29294</v>
+      </c>
       <c r="O29" s="170" t="n">
         <v>10</v>
       </c>
@@ -11519,7 +11627,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q29" s="59" t="n"/>
+      <c r="Q29" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 26 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="167" t="n">
@@ -11527,24 +11639,46 @@
       </c>
       <c r="B30" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C30" s="59" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C30" s="59" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="D30" s="168" t="n"/>
-      <c r="E30" s="168" t="n"/>
+      <c r="E30" s="168" t="n">
+        <v>46294.52878651379</v>
+      </c>
       <c r="F30" s="169">
         <f>IF(AND(D30&lt;&gt;"",E30&lt;&gt;""),(E30-D30)*24,"")</f>
         <v/>
       </c>
-      <c r="G30" s="170" t="n"/>
-      <c r="H30" s="170" t="n"/>
-      <c r="I30" s="170" t="n"/>
-      <c r="J30" s="170" t="n"/>
-      <c r="K30" s="170" t="n"/>
-      <c r="L30" s="170" t="n"/>
-      <c r="M30" s="170" t="n"/>
-      <c r="N30" s="170" t="n"/>
+      <c r="G30" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H30" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I30" s="170" t="n">
+        <v>3105</v>
+      </c>
+      <c r="J30" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="170" t="n">
+        <v>315</v>
+      </c>
+      <c r="L30" s="170" t="n">
+        <v>100</v>
+      </c>
+      <c r="M30" s="170" t="n">
+        <v>20</v>
+      </c>
+      <c r="N30" s="170" t="n">
+        <v>29991</v>
+      </c>
       <c r="O30" s="170" t="n">
         <v>10</v>
       </c>
@@ -11553,7 +11687,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q30" s="59" t="n"/>
+      <c r="Q30" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 27 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 1/10
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R593d793b649a4225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUX_CRAWL_PLAN" sheetId="2" r:id="R734f3c3038554f0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R3aed3d186d8a4483"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R7660648f363742a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_REFERENCE" sheetId="5" r:id="R38325439ffdf4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="6" r:id="Rd0cbe1e1ca9b4cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LABEL_YIELD" sheetId="7" r:id="R219cd0813e214e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="8" r:id="Rcad4a90f8ef445dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="1" r:id="R3b20a0a9c1d74925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUX_CRAWL_PLAN" sheetId="2" r:id="R4eb6a684df814fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRAWL_LOG" sheetId="3" r:id="R51d830422f17404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOCAL_REFERENCE" sheetId="4" r:id="R85a25632ed664717"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPS_REFERENCE" sheetId="5" r:id="R96c60ea1cf524250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLOT_RULES" sheetId="6" r:id="Rf427d0c06e7b4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LABEL_YIELD" sheetId="7" r:id="R44aa87b5af544636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="8" r:id="Re930dc7070c54a70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1171,7 +1171,7 @@
       </x:c>
       <x:c r="B13" s="151" t="n">
         <x:f>COUNTIFS('CRAWL_LOG'!B4:B93,"Hoàn thành")+COUNTIFS('CRAWL_LOG'!B4:B93,"Hoàn thành có lỗi")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C13" s="26" t="n"/>
       <x:c r="D13" s="26" t="n"/>
@@ -1185,7 +1185,7 @@
       </x:c>
       <x:c r="B14" s="151" t="n">
         <x:f>COUNTIF('CRAWL_LOG'!B4:B93,"Chưa chạy")</x:f>
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C14" s="26" t="n"/>
       <x:c r="D14" s="26" t="n"/>
@@ -4229,7 +4229,7 @@
       </x:c>
       <x:c r="W33" s="87" t="str">
         <x:f>'CRAWL_LOG'!B33</x:f>
-        <x:v>Chưa chạy</x:v>
+        <x:v>Hoàn thành có lỗi</x:v>
       </x:c>
       <x:c r="X33" s="95" t="inlineStr">
         <x:is>
@@ -11804,29 +11804,54 @@
         <x:v>46296</x:v>
       </x:c>
       <x:c r="B33" s="59" t="str">
-        <x:v>Chưa chạy</x:v>
-      </x:c>
-      <x:c r="C33" s="59"/>
-      <x:c r="D33" s="168"/>
-      <x:c r="E33" s="168"/>
-      <x:c r="F33" s="169"/>
-      <x:c r="G33" s="170"/>
-      <x:c r="H33" s="170"/>
-      <x:c r="I33" s="170"/>
-      <x:c r="J33" s="170"/>
-      <x:c r="K33" s="170"/>
-      <x:c r="L33" s="170"/>
-      <x:c r="M33" s="170"/>
-      <x:c r="N33" s="170"/>
+        <x:v>Hoàn thành có lỗi</x:v>
+      </x:c>
+      <x:c r="C33" s="59" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D33" s="168" t="n">
+        <x:v>46296.06282407408</x:v>
+      </x:c>
+      <x:c r="E33" s="168" t="n">
+        <x:v>46296.77693287037</x:v>
+      </x:c>
+      <x:c r="F33" s="169" t="n">
+        <x:f>IF(AND(D33&lt;&gt;"",E33&lt;&gt;""),(E33-D33)*24,"")</x:f>
+        <x:v>17.13861111109145</x:v>
+      </x:c>
+      <x:c r="G33" s="170" t="n">
+        <x:v>3540</x:v>
+      </x:c>
+      <x:c r="H33" s="170" t="n">
+        <x:v>3540</x:v>
+      </x:c>
+      <x:c r="I33" s="170" t="n">
+        <x:v>3093</x:v>
+      </x:c>
+      <x:c r="J33" s="170" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K33" s="170" t="n">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="L33" s="170" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="M33" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="N33" s="170" t="n">
+        <x:v>29357</x:v>
+      </x:c>
       <x:c r="O33" s="170" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="P33" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">local_aux</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q33" s="59"/>
+      <x:c r="P33" s="59" t="str">
+        <x:v>local_aux_backup</x:v>
+      </x:c>
+      <x:c r="Q33" s="59" t="str">
+        <x:v>Imported as run 30; SHA-256 + staging counts verified.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="167" t="n">

</xml_diff>

<commit_message>
feat: fix durable hanging
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -12017,7 +12017,7 @@
         <v>46299.02359936343</v>
       </c>
       <c r="E36" s="168" t="n">
-        <v>46299.7878555951</v>
+        <v>46299.78785559028</v>
       </c>
       <c r="F36" s="169">
         <f>IF(AND(D36&lt;&gt;"",E36&lt;&gt;""),(E36-D36)*24,"")</f>
@@ -12067,24 +12067,48 @@
       </c>
       <c r="B37" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C37" s="59" t="n"/>
-      <c r="D37" s="168" t="n"/>
-      <c r="E37" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C37" s="59" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D37" s="168" t="n">
+        <v>46300.02339822917</v>
+      </c>
+      <c r="E37" s="168" t="n">
+        <v>46300.87187777907</v>
+      </c>
       <c r="F37" s="169">
         <f>IF(AND(D37&lt;&gt;"",E37&lt;&gt;""),(E37-D37)*24,"")</f>
         <v/>
       </c>
-      <c r="G37" s="170" t="n"/>
-      <c r="H37" s="170" t="n"/>
-      <c r="I37" s="170" t="n"/>
-      <c r="J37" s="170" t="n"/>
-      <c r="K37" s="170" t="n"/>
-      <c r="L37" s="170" t="n"/>
-      <c r="M37" s="170" t="n"/>
-      <c r="N37" s="170" t="n"/>
+      <c r="G37" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H37" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I37" s="170" t="n">
+        <v>3101</v>
+      </c>
+      <c r="J37" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="170" t="n">
+        <v>289</v>
+      </c>
+      <c r="L37" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="M37" s="170" t="n">
+        <v>40</v>
+      </c>
+      <c r="N37" s="170" t="n">
+        <v>28761</v>
+      </c>
       <c r="O37" s="170" t="n">
         <v>10</v>
       </c>
@@ -12093,7 +12117,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q37" s="59" t="n"/>
+      <c r="Q37" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 34 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 10/13
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -12079,7 +12079,7 @@
         <v>46300.02339822917</v>
       </c>
       <c r="E37" s="168" t="n">
-        <v>46300.87187777907</v>
+        <v>46300.87187777778</v>
       </c>
       <c r="F37" s="169">
         <f>IF(AND(D37&lt;&gt;"",E37&lt;&gt;""),(E37-D37)*24,"")</f>
@@ -12129,24 +12129,48 @@
       </c>
       <c r="B38" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C38" s="59" t="n"/>
-      <c r="D38" s="168" t="n"/>
-      <c r="E38" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C38" s="59" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D38" s="168" t="n">
+        <v>46301.02307268519</v>
+      </c>
+      <c r="E38" s="168" t="n">
+        <v>46301.79836261574</v>
+      </c>
       <c r="F38" s="169">
         <f>IF(AND(D38&lt;&gt;"",E38&lt;&gt;""),(E38-D38)*24,"")</f>
         <v/>
       </c>
-      <c r="G38" s="170" t="n"/>
-      <c r="H38" s="170" t="n"/>
-      <c r="I38" s="170" t="n"/>
-      <c r="J38" s="170" t="n"/>
-      <c r="K38" s="170" t="n"/>
-      <c r="L38" s="170" t="n"/>
-      <c r="M38" s="170" t="n"/>
-      <c r="N38" s="170" t="n"/>
+      <c r="G38" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H38" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I38" s="170" t="n">
+        <v>3075</v>
+      </c>
+      <c r="J38" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="170" t="n">
+        <v>315</v>
+      </c>
+      <c r="L38" s="170" t="n">
+        <v>100</v>
+      </c>
+      <c r="M38" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="N38" s="170" t="n">
+        <v>29087</v>
+      </c>
       <c r="O38" s="170" t="n">
         <v>10</v>
       </c>
@@ -12155,7 +12179,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q38" s="59" t="n"/>
+      <c r="Q38" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 35 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="167" t="n">
@@ -12163,24 +12191,48 @@
       </c>
       <c r="B39" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C39" s="59" t="n"/>
-      <c r="D39" s="168" t="n"/>
-      <c r="E39" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C39" s="59" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="D39" s="168" t="n">
+        <v>46302.02296614584</v>
+      </c>
+      <c r="E39" s="168" t="n">
+        <v>46302.77321714121</v>
+      </c>
       <c r="F39" s="169">
         <f>IF(AND(D39&lt;&gt;"",E39&lt;&gt;""),(E39-D39)*24,"")</f>
         <v/>
       </c>
-      <c r="G39" s="170" t="n"/>
-      <c r="H39" s="170" t="n"/>
-      <c r="I39" s="170" t="n"/>
-      <c r="J39" s="170" t="n"/>
-      <c r="K39" s="170" t="n"/>
-      <c r="L39" s="170" t="n"/>
-      <c r="M39" s="170" t="n"/>
-      <c r="N39" s="170" t="n"/>
+      <c r="G39" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H39" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I39" s="170" t="n">
+        <v>3078</v>
+      </c>
+      <c r="J39" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="170" t="n">
+        <v>312</v>
+      </c>
+      <c r="L39" s="170" t="n">
+        <v>100</v>
+      </c>
+      <c r="M39" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="N39" s="170" t="n">
+        <v>29671</v>
+      </c>
       <c r="O39" s="170" t="n">
         <v>10</v>
       </c>
@@ -12189,7 +12241,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q39" s="59" t="n"/>
+      <c r="Q39" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 36 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="167" t="n">
@@ -12197,24 +12253,48 @@
       </c>
       <c r="B40" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C40" s="59" t="n"/>
-      <c r="D40" s="168" t="n"/>
-      <c r="E40" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C40" s="59" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="D40" s="168" t="n">
+        <v>46303.02139259259</v>
+      </c>
+      <c r="E40" s="168" t="n">
+        <v>46303.76335880787</v>
+      </c>
       <c r="F40" s="169">
         <f>IF(AND(D40&lt;&gt;"",E40&lt;&gt;""),(E40-D40)*24,"")</f>
         <v/>
       </c>
-      <c r="G40" s="170" t="n"/>
-      <c r="H40" s="170" t="n"/>
-      <c r="I40" s="170" t="n"/>
-      <c r="J40" s="170" t="n"/>
-      <c r="K40" s="170" t="n"/>
-      <c r="L40" s="170" t="n"/>
-      <c r="M40" s="170" t="n"/>
-      <c r="N40" s="170" t="n"/>
+      <c r="G40" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H40" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I40" s="170" t="n">
+        <v>3056</v>
+      </c>
+      <c r="J40" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="170" t="n">
+        <v>314</v>
+      </c>
+      <c r="L40" s="170" t="n">
+        <v>120</v>
+      </c>
+      <c r="M40" s="170" t="n">
+        <v>50</v>
+      </c>
+      <c r="N40" s="170" t="n">
+        <v>29442</v>
+      </c>
       <c r="O40" s="170" t="n">
         <v>10</v>
       </c>
@@ -12223,7 +12303,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q40" s="59" t="n"/>
+      <c r="Q40" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 37 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="167" t="n">
@@ -12231,24 +12315,48 @@
       </c>
       <c r="B41" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C41" s="59" t="n"/>
-      <c r="D41" s="168" t="n"/>
-      <c r="E41" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C41" s="59" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D41" s="168" t="n">
+        <v>46304.02179732639</v>
+      </c>
+      <c r="E41" s="168" t="n">
+        <v>46304.77693672453</v>
+      </c>
       <c r="F41" s="169">
         <f>IF(AND(D41&lt;&gt;"",E41&lt;&gt;""),(E41-D41)*24,"")</f>
         <v/>
       </c>
-      <c r="G41" s="170" t="n"/>
-      <c r="H41" s="170" t="n"/>
-      <c r="I41" s="170" t="n"/>
-      <c r="J41" s="170" t="n"/>
-      <c r="K41" s="170" t="n"/>
-      <c r="L41" s="170" t="n"/>
-      <c r="M41" s="170" t="n"/>
-      <c r="N41" s="170" t="n"/>
+      <c r="G41" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H41" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I41" s="170" t="n">
+        <v>3014</v>
+      </c>
+      <c r="J41" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="170" t="n">
+        <v>326</v>
+      </c>
+      <c r="L41" s="170" t="n">
+        <v>90</v>
+      </c>
+      <c r="M41" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N41" s="170" t="n">
+        <v>28678</v>
+      </c>
       <c r="O41" s="170" t="n">
         <v>10</v>
       </c>
@@ -12257,7 +12365,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q41" s="59" t="n"/>
+      <c r="Q41" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 38 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="167" t="n">
@@ -12265,24 +12377,48 @@
       </c>
       <c r="B42" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C42" s="59" t="n"/>
-      <c r="D42" s="168" t="n"/>
-      <c r="E42" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C42" s="59" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D42" s="168" t="n">
+        <v>46305.01922288194</v>
+      </c>
+      <c r="E42" s="168" t="n">
+        <v>46305.75559658564</v>
+      </c>
       <c r="F42" s="169">
         <f>IF(AND(D42&lt;&gt;"",E42&lt;&gt;""),(E42-D42)*24,"")</f>
         <v/>
       </c>
-      <c r="G42" s="170" t="n"/>
-      <c r="H42" s="170" t="n"/>
-      <c r="I42" s="170" t="n"/>
-      <c r="J42" s="170" t="n"/>
-      <c r="K42" s="170" t="n"/>
-      <c r="L42" s="170" t="n"/>
-      <c r="M42" s="170" t="n"/>
-      <c r="N42" s="170" t="n"/>
+      <c r="G42" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H42" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I42" s="170" t="n">
+        <v>3011</v>
+      </c>
+      <c r="J42" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="170" t="n">
+        <v>339</v>
+      </c>
+      <c r="L42" s="170" t="n">
+        <v>80</v>
+      </c>
+      <c r="M42" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N42" s="170" t="n">
+        <v>28657</v>
+      </c>
       <c r="O42" s="170" t="n">
         <v>10</v>
       </c>
@@ -12291,7 +12427,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q42" s="59" t="n"/>
+      <c r="Q42" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 39 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="167" t="n">
@@ -12299,24 +12439,48 @@
       </c>
       <c r="B43" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C43" s="59" t="n"/>
-      <c r="D43" s="168" t="n"/>
-      <c r="E43" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D43" s="168" t="n">
+        <v>46306.02048282407</v>
+      </c>
+      <c r="E43" s="168" t="n">
+        <v>46306.76039171296</v>
+      </c>
       <c r="F43" s="169">
         <f>IF(AND(D43&lt;&gt;"",E43&lt;&gt;""),(E43-D43)*24,"")</f>
         <v/>
       </c>
-      <c r="G43" s="170" t="n"/>
-      <c r="H43" s="170" t="n"/>
-      <c r="I43" s="170" t="n"/>
-      <c r="J43" s="170" t="n"/>
-      <c r="K43" s="170" t="n"/>
-      <c r="L43" s="170" t="n"/>
-      <c r="M43" s="170" t="n"/>
-      <c r="N43" s="170" t="n"/>
+      <c r="G43" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H43" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I43" s="170" t="n">
+        <v>3010</v>
+      </c>
+      <c r="J43" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="170" t="n">
+        <v>350</v>
+      </c>
+      <c r="L43" s="170" t="n">
+        <v>70</v>
+      </c>
+      <c r="M43" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N43" s="170" t="n">
+        <v>28471</v>
+      </c>
       <c r="O43" s="170" t="n">
         <v>10</v>
       </c>
@@ -12325,7 +12489,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q43" s="59" t="n"/>
+      <c r="Q43" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 40 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="167" t="n">
@@ -12333,24 +12501,48 @@
       </c>
       <c r="B44" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C44" s="59" t="n"/>
-      <c r="D44" s="168" t="n"/>
-      <c r="E44" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C44" s="59" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D44" s="168" t="n">
+        <v>46307.03053043981</v>
+      </c>
+      <c r="E44" s="168" t="n">
+        <v>46307.78793077546</v>
+      </c>
       <c r="F44" s="169">
         <f>IF(AND(D44&lt;&gt;"",E44&lt;&gt;""),(E44-D44)*24,"")</f>
         <v/>
       </c>
-      <c r="G44" s="170" t="n"/>
-      <c r="H44" s="170" t="n"/>
-      <c r="I44" s="170" t="n"/>
-      <c r="J44" s="170" t="n"/>
-      <c r="K44" s="170" t="n"/>
-      <c r="L44" s="170" t="n"/>
-      <c r="M44" s="170" t="n"/>
-      <c r="N44" s="170" t="n"/>
+      <c r="G44" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H44" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I44" s="170" t="n">
+        <v>3017</v>
+      </c>
+      <c r="J44" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="170" t="n">
+        <v>343</v>
+      </c>
+      <c r="L44" s="170" t="n">
+        <v>70</v>
+      </c>
+      <c r="M44" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N44" s="170" t="n">
+        <v>28320</v>
+      </c>
       <c r="O44" s="170" t="n">
         <v>10</v>
       </c>
@@ -12359,7 +12551,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q44" s="59" t="n"/>
+      <c r="Q44" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 41 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="167" t="n">
@@ -12367,24 +12563,48 @@
       </c>
       <c r="B45" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C45" s="59" t="n"/>
-      <c r="D45" s="168" t="n"/>
-      <c r="E45" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C45" s="59" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D45" s="168" t="n">
+        <v>46308.02002466435</v>
+      </c>
+      <c r="E45" s="168" t="n">
+        <v>46308.75924520919</v>
+      </c>
       <c r="F45" s="169">
         <f>IF(AND(D45&lt;&gt;"",E45&lt;&gt;""),(E45-D45)*24,"")</f>
         <v/>
       </c>
-      <c r="G45" s="170" t="n"/>
-      <c r="H45" s="170" t="n"/>
-      <c r="I45" s="170" t="n"/>
-      <c r="J45" s="170" t="n"/>
-      <c r="K45" s="170" t="n"/>
-      <c r="L45" s="170" t="n"/>
-      <c r="M45" s="170" t="n"/>
-      <c r="N45" s="170" t="n"/>
+      <c r="G45" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H45" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I45" s="170" t="n">
+        <v>3006</v>
+      </c>
+      <c r="J45" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="170" t="n">
+        <v>354</v>
+      </c>
+      <c r="L45" s="170" t="n">
+        <v>70</v>
+      </c>
+      <c r="M45" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N45" s="170" t="n">
+        <v>28376</v>
+      </c>
       <c r="O45" s="170" t="n">
         <v>10</v>
       </c>
@@ -12393,7 +12613,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q45" s="59" t="n"/>
+      <c r="Q45" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 42 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="167" t="n">

</xml_diff>

<commit_message>
feat: update aux crawl 14/10
</commit_message>
<xml_diff>
--- a/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
+++ b/outputs/aux-local-crawl-planner-20260901/aux_local_crawl_sampling_master.xlsx
@@ -12575,7 +12575,7 @@
         <v>46308.02002466435</v>
       </c>
       <c r="E45" s="168" t="n">
-        <v>46308.75924520919</v>
+        <v>46308.75924520833</v>
       </c>
       <c r="F45" s="169">
         <f>IF(AND(D45&lt;&gt;"",E45&lt;&gt;""),(E45-D45)*24,"")</f>
@@ -12625,24 +12625,48 @@
       </c>
       <c r="B46" s="59" t="inlineStr">
         <is>
-          <t>Chưa chạy</t>
-        </is>
-      </c>
-      <c r="C46" s="59" t="n"/>
-      <c r="D46" s="168" t="n"/>
-      <c r="E46" s="168" t="n"/>
+          <t>Hoàn thành có lỗi</t>
+        </is>
+      </c>
+      <c r="C46" s="59" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D46" s="168" t="n">
+        <v>46309.01978869213</v>
+      </c>
+      <c r="E46" s="168" t="n">
+        <v>46309.76880601719</v>
+      </c>
       <c r="F46" s="169">
         <f>IF(AND(D46&lt;&gt;"",E46&lt;&gt;""),(E46-D46)*24,"")</f>
         <v/>
       </c>
-      <c r="G46" s="170" t="n"/>
-      <c r="H46" s="170" t="n"/>
-      <c r="I46" s="170" t="n"/>
-      <c r="J46" s="170" t="n"/>
-      <c r="K46" s="170" t="n"/>
-      <c r="L46" s="170" t="n"/>
-      <c r="M46" s="170" t="n"/>
-      <c r="N46" s="170" t="n"/>
+      <c r="G46" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="H46" s="170" t="n">
+        <v>3540</v>
+      </c>
+      <c r="I46" s="170" t="n">
+        <v>3003</v>
+      </c>
+      <c r="J46" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="170" t="n">
+        <v>347</v>
+      </c>
+      <c r="L46" s="170" t="n">
+        <v>80</v>
+      </c>
+      <c r="M46" s="170" t="n">
+        <v>110</v>
+      </c>
+      <c r="N46" s="170" t="n">
+        <v>28415</v>
+      </c>
       <c r="O46" s="170" t="n">
         <v>10</v>
       </c>
@@ -12651,7 +12675,11 @@
           <t>local_aux</t>
         </is>
       </c>
-      <c r="Q46" s="59" t="n"/>
+      <c r="Q46" s="59" t="inlineStr">
+        <is>
+          <t>Scheduled run 43 terminal</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="167" t="n">

</xml_diff>